<commit_message>
Update the changes made to our app
</commit_message>
<xml_diff>
--- a/busbuddy.xlsx
+++ b/busbuddy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\philip.otieno\Desktop\busbuddy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A20C11-E319-4448-B589-08F77A9FCCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F29B518-4872-4009-8252-6C3D015EF0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="490" windowWidth="19420" windowHeight="10420" xr2:uid="{9F0F0F97-8A47-403A-8032-9D31B8DBB886}"/>
+    <workbookView xWindow="20" yWindow="620" windowWidth="19180" windowHeight="10180" xr2:uid="{9F0F0F97-8A47-403A-8032-9D31B8DBB886}"/>
   </bookViews>
   <sheets>
     <sheet name="Revenue" sheetId="1" r:id="rId1"/>
@@ -37,12 +37,6 @@
     <t>Metric</t>
   </si>
   <si>
-    <t>Target ($)</t>
-  </si>
-  <si>
-    <t>Achieved ($)</t>
-  </si>
-  <si>
     <t>% of Target</t>
   </si>
   <si>
@@ -83,6 +77,12 @@
   </si>
   <si>
     <t>Net Adds</t>
+  </si>
+  <si>
+    <t>Target (KES)</t>
+  </si>
+  <si>
+    <t>Achieved (KES)</t>
   </si>
 </sst>
 </file>
@@ -441,8 +441,8 @@
   <cols>
     <col min="1" max="1" width="26.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -457,24 +457,24 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
       </c>
       <c r="D2" s="1">
         <v>1000000</v>
@@ -483,18 +483,19 @@
         <v>238000</v>
       </c>
       <c r="F2" s="2">
+        <f>E2/D2</f>
         <v>0.23799999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
       </c>
       <c r="D3" s="1">
         <v>1000000</v>
@@ -503,18 +504,19 @@
         <v>238000</v>
       </c>
       <c r="F3" s="2">
+        <f t="shared" ref="F3:F21" si="0">E3/D3</f>
         <v>0.23799999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
       </c>
       <c r="D4" s="1">
         <v>5000000</v>
@@ -523,18 +525,19 @@
         <v>1200000</v>
       </c>
       <c r="F4" s="2">
+        <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1">
         <v>1250000</v>
@@ -543,18 +546,19 @@
         <v>300000</v>
       </c>
       <c r="F5" s="2">
+        <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D6" s="1">
         <v>1000000</v>
@@ -563,18 +567,19 @@
         <v>42000</v>
       </c>
       <c r="F6" s="2">
+        <f t="shared" si="0"/>
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
         <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
       </c>
       <c r="D7" s="1">
         <v>1000000</v>
@@ -583,18 +588,19 @@
         <v>35700</v>
       </c>
       <c r="F7" s="2">
+        <f t="shared" si="0"/>
         <v>3.5700000000000003E-2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D8" s="1">
         <v>5000000</v>
@@ -603,18 +609,19 @@
         <v>19300</v>
       </c>
       <c r="F8" s="2">
-        <v>3.8999999999999998E-3</v>
+        <f t="shared" si="0"/>
+        <v>3.8600000000000001E-3</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" s="1">
         <v>1250000</v>
@@ -623,18 +630,19 @@
         <v>15440</v>
       </c>
       <c r="F9" s="2">
-        <v>1.24E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.2352E-2</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D10" s="1">
         <v>1000000</v>
@@ -643,18 +651,19 @@
         <v>36200</v>
       </c>
       <c r="F10" s="2">
+        <f t="shared" si="0"/>
         <v>3.6200000000000003E-2</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
         <v>7</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
       </c>
       <c r="D11" s="1">
         <v>1000000</v>
@@ -663,18 +672,19 @@
         <v>30770</v>
       </c>
       <c r="F11" s="2">
-        <v>3.0800000000000001E-2</v>
+        <f t="shared" si="0"/>
+        <v>3.0769999999999999E-2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D12" s="1">
         <v>5000000</v>
@@ -683,18 +693,19 @@
         <v>27800</v>
       </c>
       <c r="F12" s="2">
-        <v>5.5999999999999999E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.5599999999999998E-3</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D13" s="1">
         <v>1250000</v>
@@ -703,18 +714,19 @@
         <v>22400</v>
       </c>
       <c r="F13" s="2">
-        <v>1.7899999999999999E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.7919999999999998E-2</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D14" s="1">
         <v>1000000</v>
@@ -723,18 +735,19 @@
         <v>36200</v>
       </c>
       <c r="F14" s="2">
+        <f t="shared" si="0"/>
         <v>3.6200000000000003E-2</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
         <v>7</v>
-      </c>
-      <c r="C15" t="s">
-        <v>9</v>
       </c>
       <c r="D15" s="1">
         <v>1000000</v>
@@ -743,18 +756,19 @@
         <v>30770</v>
       </c>
       <c r="F15" s="2">
-        <v>3.0800000000000001E-2</v>
+        <f t="shared" si="0"/>
+        <v>3.0769999999999999E-2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D16" s="1">
         <v>5000000</v>
@@ -763,18 +777,19 @@
         <v>27800</v>
       </c>
       <c r="F16" s="2">
-        <v>5.5999999999999999E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.5599999999999998E-3</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1">
         <v>1250000</v>
@@ -783,87 +798,100 @@
         <v>22400</v>
       </c>
       <c r="F17" s="2">
-        <v>1.7899999999999999E-2</v>
+        <f t="shared" si="0"/>
+        <v>1.7919999999999998E-2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D18" s="1">
+        <f>SUM(D2,D6,D10,D14)</f>
         <v>4000000</v>
       </c>
       <c r="E18" s="1">
+        <f>SUM(E2,E6,E10,E14)</f>
         <v>352400</v>
       </c>
       <c r="F18" s="2">
+        <f t="shared" si="0"/>
         <v>8.8099999999999998E-2</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
         <v>7</v>
       </c>
-      <c r="C19" t="s">
-        <v>9</v>
-      </c>
       <c r="D19" s="1">
+        <f>SUM(D3,D7,D11,D15)</f>
         <v>4000000</v>
       </c>
       <c r="E19" s="1">
+        <f>SUM(E3,E7,E11,E15)</f>
         <v>335240</v>
       </c>
       <c r="F19" s="2">
-        <v>8.3799999999999999E-2</v>
+        <f t="shared" si="0"/>
+        <v>8.3809999999999996E-2</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D20" s="1">
+        <f>SUM(D4,D8,D12,D16)</f>
         <v>20000000</v>
       </c>
       <c r="E20" s="1">
+        <f>SUM(E4,E8,E12,E16)</f>
         <v>1274900</v>
       </c>
       <c r="F20" s="2">
-        <v>6.3700000000000007E-2</v>
+        <f t="shared" si="0"/>
+        <v>6.3744999999999996E-2</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D21" s="1">
+        <f>SUM(D5,D9,D13,D17)</f>
         <v>5000000</v>
       </c>
       <c r="E21" s="1">
+        <f>SUM(E5,E9,E13,E17)</f>
         <v>360240</v>
       </c>
       <c r="F21" s="2">
-        <v>7.1999999999999995E-2</v>
+        <f t="shared" si="0"/>
+        <v>7.2048000000000001E-2</v>
       </c>
     </row>
   </sheetData>
@@ -879,7 +907,8 @@
     <col min="1" max="1" width="26.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" customWidth="1"/>
+    <col min="5" max="5" width="11.08984375" customWidth="1"/>
     <col min="6" max="6" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -894,24 +923,24 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>300</v>
@@ -920,18 +949,19 @@
         <v>22</v>
       </c>
       <c r="F2" s="2">
-        <v>0.88</v>
+        <f>E2/D2</f>
+        <v>7.3333333333333334E-2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D3">
         <v>12</v>
@@ -940,18 +970,19 @@
         <v>20</v>
       </c>
       <c r="F3" s="2">
-        <v>0.90900000000000003</v>
+        <f t="shared" ref="F3:F21" si="0">E3/D3</f>
+        <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>300</v>
@@ -960,18 +991,19 @@
         <v>15</v>
       </c>
       <c r="F4" s="2">
-        <v>0.83299999999999996</v>
+        <f t="shared" si="0"/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5">
         <v>12</v>
@@ -980,18 +1012,19 @@
         <v>12</v>
       </c>
       <c r="F5" s="2">
-        <v>0.8</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>300</v>
@@ -1000,18 +1033,19 @@
         <v>26</v>
       </c>
       <c r="F6" s="2">
-        <v>1.04</v>
+        <f t="shared" si="0"/>
+        <v>8.666666666666667E-2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7">
         <v>12</v>
@@ -1020,18 +1054,19 @@
         <v>22</v>
       </c>
       <c r="F7" s="2">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>1.8333333333333333</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8">
         <v>300</v>
@@ -1040,18 +1075,19 @@
         <v>15</v>
       </c>
       <c r="F8" s="2">
-        <v>0.83299999999999996</v>
+        <f t="shared" si="0"/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9">
         <v>12</v>
@@ -1060,18 +1096,19 @@
         <v>11</v>
       </c>
       <c r="F9" s="2">
-        <v>0.73299999999999998</v>
+        <f t="shared" si="0"/>
+        <v>0.91666666666666663</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>300</v>
@@ -1080,18 +1117,19 @@
         <v>24</v>
       </c>
       <c r="F10" s="2">
-        <v>0.8</v>
+        <f t="shared" si="0"/>
+        <v>0.08</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11">
         <v>12</v>
@@ -1100,18 +1138,19 @@
         <v>20</v>
       </c>
       <c r="F11" s="2">
-        <v>0.8</v>
+        <f t="shared" si="0"/>
+        <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>300</v>
@@ -1120,18 +1159,19 @@
         <v>15</v>
       </c>
       <c r="F12" s="2">
-        <v>0.75</v>
+        <f t="shared" si="0"/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D13">
         <v>12</v>
@@ -1140,18 +1180,19 @@
         <v>10</v>
       </c>
       <c r="F13" s="2">
-        <v>0.66700000000000004</v>
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <v>300</v>
@@ -1160,18 +1201,19 @@
         <v>24</v>
       </c>
       <c r="F14" s="2">
-        <v>0.8</v>
+        <f t="shared" si="0"/>
+        <v>0.08</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D15">
         <v>12</v>
@@ -1180,18 +1222,19 @@
         <v>20</v>
       </c>
       <c r="F15" s="2">
-        <v>0.8</v>
+        <f t="shared" si="0"/>
+        <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D16">
         <v>300</v>
@@ -1200,18 +1243,19 @@
         <v>15</v>
       </c>
       <c r="F16" s="2">
-        <v>0.75</v>
+        <f t="shared" si="0"/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D17">
         <v>12</v>
@@ -1220,87 +1264,100 @@
         <v>10</v>
       </c>
       <c r="F17" s="2">
-        <v>0.66700000000000004</v>
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D18">
+        <f>SUM(D2,D6,D10,D14)</f>
         <v>1200</v>
       </c>
       <c r="E18">
+        <f>SUM(E2,E6,E10,E14)</f>
         <v>96</v>
       </c>
       <c r="F18" s="2">
-        <v>0.66700000000000004</v>
+        <f>E18/D18</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D19">
+        <f>SUM(D3,D7,D11,D15)</f>
         <v>48</v>
       </c>
       <c r="E19">
+        <f>SUM(E3,E7,E11,E15)</f>
         <v>82</v>
       </c>
       <c r="F19" s="2">
-        <v>0.66700000000000004</v>
+        <f>E19/D19</f>
+        <v>1.7083333333333333</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D20">
+        <f>SUM(D4,D8,D12,D16)</f>
         <v>1200</v>
       </c>
       <c r="E20">
+        <f>SUM(E4,E8,E12,E16)</f>
         <v>60</v>
       </c>
       <c r="F20" s="2">
-        <v>0.66700000000000004</v>
+        <f t="shared" si="0"/>
+        <v>0.05</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D21">
+        <f>SUM(D5,D9,D13,D17)</f>
         <v>48</v>
       </c>
       <c r="E21">
+        <f>SUM(E5,E9,E13,E17)</f>
         <v>43</v>
       </c>
       <c r="F21" s="2">
-        <v>0.66700000000000004</v>
+        <f t="shared" si="0"/>
+        <v>0.89583333333333337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>